<commit_message>
Update paths in the evaluation script for ectopic beats detection
</commit_message>
<xml_diff>
--- a/0_SELECT_ZIVE_DATA_2023/AnotacijosLogai/09_Anotacijos_logai/09_Anotavimo_logas.xlsx
+++ b/0_SELECT_ZIVE_DATA_2023/AnotacijosLogai/09_Anotacijos_logai/09_Anotavimo_logas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\kesju\DI\2025_ZIVEO\PROJECT_TRAIN_UNET\0_SELECT_ZIVE_DATA_2023\AnotacijosLogai\09_Anotacijos_logai\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF394C77-AE28-4C97-9F28-62F63A32802A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9340D20B-B994-40A2-9FF3-7770663E4ACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -705,10 +705,9 @@
       <c r="G2" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="H2" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="I2" s="4"/>
+      <c r="I2" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="J2" s="4"/>
       <c r="K2" s="13" t="s">
         <v>3</v>
@@ -743,10 +742,10 @@
       <c r="G3" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="H3" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="I3" s="4"/>
+      <c r="H3" s="4"/>
+      <c r="I3" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="J3" s="4"/>
       <c r="K3" s="13" t="s">
         <v>7</v>
@@ -779,10 +778,9 @@
       <c r="G4" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="H4" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="I4" s="4"/>
+      <c r="I4" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="J4" s="4"/>
       <c r="K4" s="13"/>
       <c r="L4" t="s">
@@ -813,10 +811,9 @@
       <c r="G5" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="H5" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="I5" s="4"/>
+      <c r="I5" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="J5" s="4"/>
       <c r="K5" s="13" t="s">
         <v>12</v>
@@ -944,10 +941,9 @@
       <c r="G9" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="H9" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="I9" s="8"/>
+      <c r="I9" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="J9" s="8"/>
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.35">
@@ -966,10 +962,9 @@
       <c r="G10" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="H10" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="I10" s="8"/>
+      <c r="I10" s="4" t="b">
+        <v>1</v>
+      </c>
       <c r="J10" s="8"/>
       <c r="N10" t="s">
         <v>42</v>

</xml_diff>